<commit_message>
update: updated User folder for testing
</commit_message>
<xml_diff>
--- a/User/reservations.xlsx
+++ b/User/reservations.xlsx
@@ -478,18 +478,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>customer1</t>
+          <t>John</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-06-07</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="F2" t="n">

</xml_diff>